<commit_message>
lab01 - specified where problems where found (line, page)
</commit_message>
<xml_diff>
--- a/docs/Lab01/Solutions/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Solutions/Lab01_ReviewReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UBB\semestrul 6\VVSS\MyDrinkShop\docs\Lab01\Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94AD5BBA-1E89-4C49-A64D-032769EB2F6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8087F37A-CD7E-4AEC-879E-0A936156EA55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-408" yWindow="1752" windowWidth="19752" windowHeight="8880" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1752" windowWidth="19752" windowHeight="8880" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="64">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -210,6 +210,24 @@
   </si>
   <si>
     <t>DrinkShopController + liste (productList, retetaList, etc.). Layering neclar. Solutie: separare pe layers, controller doar apeleaza DrinkShopService (DTO/ViewModel), business-ul ramane in Service.</t>
+  </si>
+  <si>
+    <t>pag1 / cerinte functionale pct. 6</t>
+  </si>
+  <si>
+    <t>pag1 / cerinte functionale pct. 1</t>
+  </si>
+  <si>
+    <t>pag1 / cerinte non-functionale pct. 3</t>
+  </si>
+  <si>
+    <t>pag1 / cerinte functionale pct. 8</t>
+  </si>
+  <si>
+    <t>pag1 / cerinte functionale pct. 1, 6</t>
+  </si>
+  <si>
+    <t>nothing about errors</t>
   </si>
 </sst>
 </file>
@@ -408,7 +426,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -439,6 +457,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -481,7 +500,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -807,19 +828,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -832,10 +853,10 @@
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="36" t="s">
+      <c r="I3" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="36">
+      <c r="J3" s="22">
         <v>232</v>
       </c>
     </row>
@@ -843,17 +864,17 @@
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="25"/>
+      <c r="E4" s="26"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="36" t="s">
+      <c r="I4" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="J4" s="36">
+      <c r="J4" s="22">
         <v>232</v>
       </c>
     </row>
@@ -861,17 +882,17 @@
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="27"/>
+      <c r="E5" s="28"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="36" t="s">
+      <c r="I5" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="J5" s="36">
+      <c r="J5" s="22">
         <v>232</v>
       </c>
     </row>
@@ -880,19 +901,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="E6" s="22"/>
+      <c r="E6" s="23"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="22" t="s">
+      <c r="D7" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E7" s="22"/>
+      <c r="E7" s="23"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -915,7 +936,9 @@
       <c r="C10" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="1"/>
+      <c r="D10" s="37" t="s">
+        <v>58</v>
+      </c>
       <c r="E10" s="2" t="s">
         <v>44</v>
       </c>
@@ -928,7 +951,9 @@
       <c r="C11" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="1"/>
+      <c r="D11" s="37" t="s">
+        <v>62</v>
+      </c>
       <c r="E11" s="2" t="s">
         <v>38</v>
       </c>
@@ -941,7 +966,9 @@
       <c r="C12" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="1"/>
+      <c r="D12" s="37" t="s">
+        <v>60</v>
+      </c>
       <c r="E12" s="2" t="s">
         <v>39</v>
       </c>
@@ -954,7 +981,9 @@
       <c r="C13" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D13" s="1"/>
+      <c r="D13" s="37" t="s">
+        <v>61</v>
+      </c>
       <c r="E13" s="2" t="s">
         <v>40</v>
       </c>
@@ -967,7 +996,9 @@
       <c r="C14" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="1"/>
+      <c r="D14" s="37" t="s">
+        <v>59</v>
+      </c>
       <c r="E14" s="2" t="s">
         <v>41</v>
       </c>
@@ -980,12 +1011,14 @@
       <c r="C15" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D15" s="1"/>
+      <c r="D15" s="37" t="s">
+        <v>63</v>
+      </c>
       <c r="E15" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -993,7 +1026,9 @@
       <c r="C16" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D16" s="1"/>
+      <c r="D16" s="37" t="s">
+        <v>60</v>
+      </c>
       <c r="E16" s="2" t="s">
         <v>43</v>
       </c>
@@ -1006,7 +1041,9 @@
       <c r="C17" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D17" s="3"/>
+      <c r="D17" s="37" t="s">
+        <v>60</v>
+      </c>
       <c r="E17" s="2" t="s">
         <v>45</v>
       </c>
@@ -1125,19 +1162,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1150,10 +1187,10 @@
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="36" t="s">
+      <c r="I3" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="36">
+      <c r="J3" s="22">
         <v>232</v>
       </c>
     </row>
@@ -1161,17 +1198,17 @@
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="28"/>
+      <c r="E4" s="29"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="36" t="s">
+      <c r="I4" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="J4" s="36">
+      <c r="J4" s="22">
         <v>232</v>
       </c>
     </row>
@@ -1179,17 +1216,17 @@
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="30"/>
+      <c r="E5" s="31"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="36" t="s">
+      <c r="I5" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="J5" s="36">
+      <c r="J5" s="22">
         <v>232</v>
       </c>
     </row>
@@ -1198,19 +1235,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="E6" s="22"/>
+      <c r="E6" s="23"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="22" t="s">
+      <c r="D7" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E7" s="22"/>
+      <c r="E7" s="23"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -1440,19 +1477,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1465,10 +1502,10 @@
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="36" t="s">
+      <c r="I3" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="36">
+      <c r="J3" s="22">
         <v>232</v>
       </c>
     </row>
@@ -1476,17 +1513,17 @@
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="31" t="s">
+      <c r="D4" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="31"/>
+      <c r="E4" s="32"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="36" t="s">
+      <c r="I4" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="J4" s="36">
+      <c r="J4" s="22">
         <v>232</v>
       </c>
     </row>
@@ -1494,17 +1531,17 @@
       <c r="C5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="D5" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="33"/>
+      <c r="E5" s="34"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="36" t="s">
+      <c r="I5" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="J5" s="36">
+      <c r="J5" s="22">
         <v>232</v>
       </c>
     </row>
@@ -1513,15 +1550,15 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -1770,19 +1807,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1795,10 +1832,10 @@
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="36" t="s">
+      <c r="I3" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="36">
+      <c r="J3" s="22">
         <v>232</v>
       </c>
     </row>
@@ -1806,15 +1843,15 @@
       <c r="C4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="36" t="s">
+      <c r="I4" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="J4" s="36">
+      <c r="J4" s="22">
         <v>232</v>
       </c>
     </row>
@@ -1822,15 +1859,15 @@
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="36" t="s">
+      <c r="I5" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="J5" s="36">
+      <c r="J5" s="22">
         <v>232</v>
       </c>
     </row>
@@ -1839,8 +1876,8 @@
       <c r="C6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
       <c r="F6" s="20"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -2070,11 +2107,11 @@
       <c r="F30" s="2"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C32" s="34" t="s">
+      <c r="C32" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="35"/>
-      <c r="E32" s="35"/>
+      <c r="D32" s="36"/>
+      <c r="E32" s="36"/>
       <c r="F32" s="18"/>
     </row>
     <row r="35" spans="6:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Rezolvare 1.3 si 2.3 din Lab01
</commit_message>
<xml_diff>
--- a/docs/Lab01/Solutions/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Solutions/Lab01_ReviewReport.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UBB\semestrul 6\VVSS\MyDrinkShop\docs\Lab01\Solutions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexcostan/Documents/FACULTATE/SEM2/VVSS/LAB1/vvss-project/docs/Lab01/Solutions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8087F37A-CD7E-4AEC-879E-0A936156EA55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4A759F3-6B38-DE43-B98B-8572FF0B010A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1752" windowWidth="19752" windowHeight="8880" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="16960" tabRatio="650" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="76">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -228,6 +228,42 @@
   </si>
   <si>
     <t>nothing about errors</t>
+  </si>
+  <si>
+    <t>Costan Alex-Ionut</t>
+  </si>
+  <si>
+    <t>C05</t>
+  </si>
+  <si>
+    <t>Codul presupune ca metoda findOne returneaza mereu un obiect valid, dar in realitate aceasta metoda returneaza null daca nu se gaseste obiectul cu ID dat, existand riscul sa se declanseze o eroare de tip NullPointerException. Trebuie mereu sa se verifice daca s-a gasit ceva inainte sa se utilizeze rezultatul</t>
+  </si>
+  <si>
+    <t>C01</t>
+  </si>
+  <si>
+    <t>StocValidator - linia 24</t>
+  </si>
+  <si>
+    <t>Logica de decizie este inadecvata deoarece se trateaza o conditie de bussiness ca fiind o eroare de validare; validarea ar trebui sa asigure consistenta datelor (ex: sa nu fie pret/cantitate negative), nu sa impuna constrangeri asupra procesului de vanzare</t>
+  </si>
+  <si>
+    <t>C06</t>
+  </si>
+  <si>
+    <t>Codul aplica Double direct pe textul introdus de utilizator, fara a verifica daca acesta este format exclusiv din cifre; daca se lasa campul gol sau se introduc caractere non-numerice, programul arunca exceptia NumberFormatException; ar trebui sa se utilizeze un bloc try-catch</t>
+  </si>
+  <si>
+    <t>DrinkShopController - 132</t>
+  </si>
+  <si>
+    <t>DrinkShopController - 182</t>
+  </si>
+  <si>
+    <t>Generare incorecta de ID. Codul ia numarul total de elemente la care adauga 1, ceea ce e gresit, deoarece nu garantam unicitatea id-urilor (ex: avem id urile 1, 2, 3; stergem obiectul cu id 2, deci mai avem 2 obiecte; cream unul nou, automat primeste id 3 care e deja existent.). ar trebui sa luam cel mai mare id, la care ii adaugam 1</t>
+  </si>
+  <si>
+    <t>OrderService - linia 43</t>
   </si>
 </sst>
 </file>
@@ -426,7 +462,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -458,6 +494,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -500,9 +539,14 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -811,36 +855,36 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="6"/>
-    <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
-    <col min="3" max="4" width="16.21875" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.44140625" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.88671875" style="6"/>
+    <col min="1" max="1" width="8.83203125" style="6"/>
+    <col min="2" max="2" width="12.1640625" style="6" customWidth="1"/>
+    <col min="3" max="4" width="16.1640625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="41.5" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.83203125" style="6"/>
     <col min="9" max="9" width="21" style="6" customWidth="1"/>
-    <col min="10" max="10" width="14.44140625" style="6" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="6"/>
+    <col min="10" max="10" width="14.5" style="6" customWidth="1"/>
+    <col min="11" max="16384" width="8.83203125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B2" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -849,7 +893,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
@@ -860,14 +904,14 @@
         <v>232</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="26"/>
+      <c r="E4" s="27"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -878,14 +922,14 @@
         <v>232</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="27" t="s">
+      <c r="D5" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="28"/>
+      <c r="E5" s="29"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -896,26 +940,26 @@
         <v>232</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="23" t="s">
+      <c r="D6" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="E6" s="23"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E6" s="24"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="E7" s="23"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E7" s="24"/>
+    </row>
+    <row r="9" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -929,21 +973,21 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="B10" s="3">
         <v>1</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="37" t="s">
+      <c r="D10" s="23" t="s">
         <v>58</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -951,14 +995,14 @@
       <c r="C11" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="37" t="s">
+      <c r="D11" s="23" t="s">
         <v>62</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B25" si="0">B11+1</f>
         <v>3</v>
@@ -966,14 +1010,14 @@
       <c r="C12" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="37" t="s">
+      <c r="D12" s="23" t="s">
         <v>60</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -981,14 +1025,14 @@
       <c r="C13" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D13" s="37" t="s">
+      <c r="D13" s="23" t="s">
         <v>61</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -996,14 +1040,14 @@
       <c r="C14" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="37" t="s">
+      <c r="D14" s="23" t="s">
         <v>59</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1011,14 +1055,14 @@
       <c r="C15" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D15" s="37" t="s">
+      <c r="D15" s="23" t="s">
         <v>63</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1026,14 +1070,14 @@
       <c r="C16" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D16" s="37" t="s">
+      <c r="D16" s="23" t="s">
         <v>60</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1041,20 +1085,20 @@
       <c r="C17" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D17" s="37" t="s">
+      <c r="D17" s="23" t="s">
         <v>60</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1063,7 +1107,7 @@
       <c r="D19" s="3"/>
       <c r="E19" s="15"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1072,7 +1116,7 @@
       <c r="D20" s="3"/>
       <c r="E20" s="15"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1081,7 +1125,7 @@
       <c r="D21" s="3"/>
       <c r="E21" s="15"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1090,7 +1134,7 @@
       <c r="D22" s="3"/>
       <c r="E22" s="15"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1099,7 +1143,7 @@
       <c r="D23" s="3"/>
       <c r="E23" s="15"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1108,7 +1152,7 @@
       <c r="D24" s="3"/>
       <c r="E24" s="15"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1117,7 +1161,7 @@
       <c r="D25" s="3"/>
       <c r="E25" s="15"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.2">
       <c r="C27" s="11" t="s">
         <v>8</v>
       </c>
@@ -1146,35 +1190,35 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J28"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="6"/>
-    <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
-    <col min="3" max="4" width="16.21875" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.44140625" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.88671875" style="6"/>
-    <col min="9" max="9" width="22.109375" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="6"/>
+    <col min="1" max="1" width="8.83203125" style="6"/>
+    <col min="2" max="2" width="12.1640625" style="6" customWidth="1"/>
+    <col min="3" max="4" width="16.1640625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="41.5" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.83203125" style="6"/>
+    <col min="9" max="9" width="22.1640625" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.83203125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B2" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1183,7 +1227,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
@@ -1194,14 +1238,14 @@
         <v>232</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="29"/>
+      <c r="E4" s="30"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -1212,14 +1256,14 @@
         <v>232</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="31"/>
+      <c r="E5" s="32"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1230,26 +1274,26 @@
         <v>232</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="23" t="s">
+      <c r="D6" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="E6" s="23"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E6" s="24"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="E7" s="23"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E7" s="24"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1263,7 +1307,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1277,7 +1321,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -1292,7 +1336,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B26" si="0">B11+1</f>
         <v>3</v>
@@ -1307,7 +1351,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1316,7 +1360,7 @@
       <c r="D13" s="1"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1325,7 +1369,7 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1334,7 +1378,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1343,7 +1387,7 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1352,7 +1396,7 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1361,7 +1405,7 @@
       <c r="D18" s="1"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1370,7 +1414,7 @@
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1379,7 +1423,7 @@
       <c r="D20" s="1"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1388,7 +1432,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1397,7 +1441,7 @@
       <c r="D22" s="1"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1406,7 +1450,7 @@
       <c r="D23" s="1"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1415,7 +1459,7 @@
       <c r="D24" s="1"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1424,7 +1468,7 @@
       <c r="D25" s="1"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1433,7 +1477,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.2">
       <c r="C28" s="11" t="s">
         <v>8</v>
       </c>
@@ -1460,36 +1504,36 @@
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="6"/>
-    <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.21875" style="6" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="6"/>
+    <col min="2" max="2" width="12.1640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.1640625" style="6" customWidth="1"/>
     <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.44140625" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.88671875" style="6"/>
-    <col min="9" max="9" width="26.77734375" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="6"/>
+    <col min="5" max="5" width="41.5" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.83203125" style="6"/>
+    <col min="9" max="9" width="26.83203125" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.83203125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B2" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1498,7 +1542,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
@@ -1509,14 +1553,14 @@
         <v>232</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="32"/>
+      <c r="E4" s="33"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -1527,14 +1571,14 @@
         <v>232</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="33" t="s">
+      <c r="D5" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="34"/>
+      <c r="E5" s="35"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1545,224 +1589,252 @@
         <v>232</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D6" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" s="24"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B9" s="10" t="s">
+      <c r="D7" s="38">
+        <v>46095</v>
+      </c>
+      <c r="E7" s="24"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B9" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="40" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B10" s="3">
+    <row r="10" spans="1:10" ht="112" x14ac:dyDescent="0.2">
+      <c r="B10" s="41">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B11" s="3">
+      <c r="C10" s="39" t="s">
+        <v>65</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="80" x14ac:dyDescent="0.2">
+      <c r="B11" s="41">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B12" s="3">
+      <c r="C11" s="39" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" s="39" t="s">
+        <v>68</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="96" x14ac:dyDescent="0.2">
+      <c r="B12" s="41">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B13" s="3">
+      <c r="C12" s="39" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="112" x14ac:dyDescent="0.2">
+      <c r="B13" s="41">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B14" s="3">
+      <c r="C13" s="39" t="s">
+        <v>67</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B14" s="41">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
+      <c r="C14" s="39"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B15" s="3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B15" s="41">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="1"/>
+      <c r="C15" s="39"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B16" s="3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B16" s="41">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="1"/>
+      <c r="C16" s="39"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B17" s="3">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B17" s="41">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="1"/>
+      <c r="C17" s="39"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B18" s="3">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B18" s="41">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="1"/>
+      <c r="C18" s="39"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B19" s="3">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B19" s="41">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="39"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B20" s="3">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B20" s="41">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="1"/>
+      <c r="C20" s="39"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B21" s="3">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B21" s="41">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
+      <c r="C21" s="39"/>
+      <c r="D21" s="39"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B22" s="3">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B22" s="41">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="1"/>
+      <c r="C22" s="39"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B23" s="3">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B23" s="41">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="1"/>
+      <c r="C23" s="39"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B24" s="3">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B24" s="41">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="1"/>
+      <c r="C24" s="39"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B25" s="3">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B25" s="41">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="1"/>
+      <c r="C25" s="39"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B26" s="3">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B26" s="41">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
+      <c r="C26" s="39"/>
+      <c r="D26" s="39"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B27" s="3">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B27" s="41">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="1"/>
+      <c r="C27" s="39"/>
       <c r="D27" s="2"/>
-      <c r="E27" s="1"/>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B28" s="3">
+      <c r="E27" s="39"/>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B28" s="41">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C28" s="1"/>
+      <c r="C28" s="39"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B29" s="3">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B29" s="41">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C29" s="1"/>
+      <c r="C29" s="39"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B30" s="3">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B30" s="41">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C30" s="1"/>
+      <c r="C30" s="39"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
       <c r="C32" s="11" t="s">
         <v>8</v>
       </c>
@@ -1789,37 +1861,37 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:J35"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="6"/>
-    <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.21875" style="6" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="6"/>
+    <col min="2" max="2" width="12.1640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.1640625" style="6" customWidth="1"/>
     <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="23.88671875" style="6" customWidth="1"/>
+    <col min="5" max="5" width="23.83203125" style="6" customWidth="1"/>
     <col min="6" max="6" width="16.6640625" style="6" customWidth="1"/>
-    <col min="7" max="8" width="8.88671875" style="6"/>
-    <col min="9" max="9" width="26.77734375" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="6"/>
+    <col min="7" max="8" width="8.83203125" style="6"/>
+    <col min="9" max="9" width="26.83203125" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.83203125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B2" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1828,7 +1900,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
@@ -1839,12 +1911,12 @@
         <v>232</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -1855,12 +1927,12 @@
         <v>232</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1871,16 +1943,16 @@
         <v>232</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
       <c r="F6" s="20"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1897,7 +1969,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1906,7 +1978,7 @@
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -1916,7 +1988,7 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
@@ -1926,7 +1998,7 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1936,7 +2008,7 @@
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1946,7 +2018,7 @@
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1956,7 +2028,7 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1966,7 +2038,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1976,7 +2048,7 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1986,7 +2058,7 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1996,7 +2068,7 @@
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2006,7 +2078,7 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -2016,7 +2088,7 @@
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -2026,7 +2098,7 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2036,7 +2108,7 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2046,7 +2118,7 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -2056,7 +2128,7 @@
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -2066,7 +2138,7 @@
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2076,7 +2148,7 @@
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -2086,7 +2158,7 @@
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -2096,7 +2168,7 @@
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B30" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -2106,15 +2178,15 @@
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C32" s="35" t="s">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="C32" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="36"/>
-      <c r="E32" s="36"/>
+      <c r="D32" s="37"/>
+      <c r="E32" s="37"/>
       <c r="F32" s="18"/>
     </row>
-    <row r="35" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F35" s="21"/>
     </row>
   </sheetData>

</xml_diff>